<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-07-22)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9298245614035088</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.211494616704504</v>
+        <v>1.230936658375462</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>2.909810215614418</v>
+        <v>2.965699092143766</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.4011466028965043</v>
+        <v>0.3948538299914004</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.01500000000000012</v>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8193981481481482</v>
+        <v>0.8214035087719298</v>
       </c>
     </row>
     <row r="3">
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>810</v>
+        <v>823</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9950617283950617</v>
+        <v>0.9951397326852977</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.9244216055834175</v>
+        <v>0.942253938858188</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1.845107080764028</v>
+        <v>1.872624840485766</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.2134078865496956</v>
+        <v>0.2117228565766469</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.05833537351557738</v>
@@ -568,7 +568,7 @@
         <v>17</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9853623456790124</v>
+        <v>0.9853809234507899</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9949324324324325</v>
+        <v>0.9950248756218906</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.6432573461737613</v>
+        <v>0.6554387811951277</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.618144640085836</v>
+        <v>1.634704427506083</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.164140706524158</v>
+        <v>0.1623543426650389</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.05450205413924314</v>
@@ -599,7 +599,7 @@
         <v>11</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9862863175675675</v>
+        <v>0.986337479270315</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.3809635051512486</v>
+        <v>0.3857104020819992</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.392274030837791</v>
+        <v>1.398234154216364</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1101630143863725</v>
+        <v>0.1080651026370896</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.01386579723875603</v>
@@ -630,7 +630,7 @@
         <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9872609375</v>
+        <v>0.9872746913580247</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9919786096256684</v>
+        <v>0.9895013123359579</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.592458121855753</v>
+        <v>1.616647060457461</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3.688480226999131</v>
+        <v>3.773057879979477</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.5100956653419606</v>
+        <v>0.5015466056877711</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.02127438923763525</v>
       </c>
       <c r="H6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.963024064171123</v>
+        <v>0.9624593175853019</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-19T09:06:05+00:00 · arquivo de 1718 dias-cidade (~95 dias corridos) · 18 cidades</t>
+          <t>Atualizado em 2026-07-22T09:07:15+00:00 · arquivo de 1772 dias-cidade (~98 dias corridos) · 18 cidades</t>
         </is>
       </c>
     </row>
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.04118168176312127</v>
+        <v>0.02618168176312127</v>
       </c>
     </row>
     <row r="11">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.1111358245807016</v>
+        <v>0.131617752291545</v>
       </c>
     </row>
     <row r="12">
@@ -1011,13 +1011,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.02137283006848223</v>
+        <v>0.03533294402859619</v>
       </c>
     </row>
     <row r="16">
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.05952500982236602</v>
+        <v>0.06251162156283976</v>
       </c>
     </row>
     <row r="20">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.1666445629886013</v>
+        <v>0.1672481847189836</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.04639044076973562</v>
+        <v>0.03139044076973562</v>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.1366634849983473</v>
+        <v>0.1571454127091907</v>
       </c>
     </row>
     <row r="29">
@@ -1347,13 +1347,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.08584108705952805</v>
+        <v>0.08639412878904036</v>
       </c>
     </row>
     <row r="32">
@@ -1368,13 +1368,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.02896133565011405</v>
+        <v>0.0435250713406103</v>
       </c>
     </row>
     <row r="33">
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>943</v>
+        <v>964</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8727</v>
+        <v>0.8754999999999999</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.992</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="3">
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>952</v>
+        <v>973</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8666</v>
+        <v>0.8695000000000001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9949</v>
+        <v>0.9946</v>
       </c>
     </row>
     <row r="4">
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>982</v>
+        <v>1008</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8737</v>
+        <v>0.877</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9953</v>
+        <v>0.9949</v>
       </c>
     </row>
     <row r="5">
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>976</v>
+        <v>998</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8658</v>
+        <v>0.8687</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9964</v>
+        <v>0.9962</v>
       </c>
     </row>
     <row r="6">
@@ -1511,13 +1511,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>996</v>
+        <v>1021</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8464</v>
+        <v>0.8501</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9974</v>
+        <v>0.9972</v>
       </c>
     </row>
     <row r="7">
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>969</v>
+        <v>990</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8576</v>
+        <v>0.8606</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.997</v>
+        <v>0.9967</v>
       </c>
     </row>
     <row r="8">
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>993</v>
+        <v>1015</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8439</v>
+        <v>0.8473000000000001</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9968</v>
+        <v>0.9965000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -1559,13 +1559,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>926</v>
+        <v>948</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8985</v>
+        <v>0.8987000000000001</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9912</v>
+        <v>0.9906</v>
       </c>
     </row>
     <row r="10">
@@ -1575,13 +1575,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>902</v>
+        <v>920</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8725000000000001</v>
+        <v>0.875</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9908</v>
       </c>
     </row>
     <row r="11">
@@ -1591,10 +1591,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>937</v>
+        <v>962</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.9274</v>
+        <v>0.9293</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>0.9935</v>
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>925</v>
+        <v>945</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.9124</v>
+        <v>0.9132</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9878</v>
+        <v>0.9873</v>
       </c>
     </row>
     <row r="13">
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>916</v>
+        <v>938</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.9016999999999999</v>
+        <v>0.903</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9873</v>
+        <v>0.987</v>
       </c>
     </row>
     <row r="14">
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>914</v>
+        <v>938</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8731</v>
+        <v>0.8763</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9928</v>
+        <v>0.9925</v>
       </c>
     </row>
     <row r="15">
@@ -1655,13 +1655,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>951</v>
+        <v>974</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8686</v>
+        <v>0.8717</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9938</v>
+        <v>0.9936</v>
       </c>
     </row>
     <row r="16">
@@ -1671,10 +1671,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>935</v>
+        <v>956</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8738</v>
+        <v>0.8766</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0.9902</v>
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>900</v>
+        <v>920</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.9167</v>
+        <v>0.9185</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9916</v>
+        <v>0.9915</v>
       </c>
     </row>
     <row r="18">
@@ -1703,13 +1703,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>971</v>
+        <v>993</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8599</v>
+        <v>0.863</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9966</v>
+        <v>0.9963</v>
       </c>
     </row>
     <row r="19">
@@ -1719,13 +1719,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>971</v>
+        <v>998</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8847</v>
+        <v>0.8868</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9913</v>
+        <v>0.9912</v>
       </c>
     </row>
   </sheetData>
@@ -1789,19 +1789,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1372</v>
+        <v>0.1351</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1372</v>
+        <v>0.1351</v>
       </c>
       <c r="D2" t="n">
-        <v>1.2781</v>
+        <v>1.4556</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.6977</v>
+        <v>-0.393</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2158</v>
+        <v>0.1874</v>
       </c>
     </row>
     <row r="3">
@@ -1811,16 +1811,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1305</v>
+        <v>0.1291</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1207</v>
+        <v>0.1197</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0036</v>
+        <v>0.0034</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0469</v>
+        <v>1.051</v>
       </c>
       <c r="F3" t="n">
         <v>0.08069999999999999</v>
@@ -1833,19 +1833,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0445</v>
+        <v>0.0442</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0386</v>
+        <v>0.0385</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1218</v>
+        <v>0.1216</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9756</v>
+        <v>0.9785</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0609</v>
+        <v>0.0608</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-19T09:06:05+00:00</t>
+          <t>2026-07-22T09:07:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1718</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="3">
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>